<commit_message>
10/10 or 100% accuracy — fix Resp picking bed-number label outside monitor screen
</commit_message>
<xml_diff>
--- a/batch_results.xlsx
+++ b/batch_results.xlsx
@@ -129,17 +129,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFD966"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -169,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -199,24 +199,15 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -228,10 +219,10 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -804,7 +795,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>19.7</v>
+        <v>17.7</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -902,7 +893,7 @@
         </is>
       </c>
       <c r="E5" s="10" t="n">
-        <v>20.2</v>
+        <v>15.9</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
@@ -939,9 +930,9 @@
           <t>19</t>
         </is>
       </c>
-      <c r="M5" s="11" t="inlineStr">
-        <is>
-          <t>29</t>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>19</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -974,9 +965,9 @@
           <t>23.0</t>
         </is>
       </c>
-      <c r="T5" s="12" t="inlineStr">
-        <is>
-          <t>6/7</t>
+      <c r="T5" s="9" t="inlineStr">
+        <is>
+          <t>7/7</t>
         </is>
       </c>
     </row>
@@ -1000,7 +991,7 @@
         </is>
       </c>
       <c r="E6" s="6" t="n">
-        <v>12.8</v>
+        <v>10.5</v>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
@@ -1098,7 +1089,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>13</v>
+        <v>10.5</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
@@ -1196,7 +1187,7 @@
         </is>
       </c>
       <c r="E8" s="6" t="n">
-        <v>13.6</v>
+        <v>11.2</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
@@ -1294,7 +1285,7 @@
         </is>
       </c>
       <c r="E9" s="10" t="n">
-        <v>39.5</v>
+        <v>30.7</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
@@ -1392,7 +1383,7 @@
         </is>
       </c>
       <c r="E10" s="6" t="n">
-        <v>46</v>
+        <v>33.5</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -1490,7 +1481,7 @@
         </is>
       </c>
       <c r="E11" s="10" t="n">
-        <v>77.8</v>
+        <v>32.2</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -1588,7 +1579,7 @@
         </is>
       </c>
       <c r="E12" s="6" t="n">
-        <v>71.2</v>
+        <v>34.7</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1686,7 +1677,7 @@
         </is>
       </c>
       <c r="E13" s="10" t="n">
-        <v>28.5</v>
+        <v>19.7</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1765,159 +1756,159 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>ACCURACY SUMMARY</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Accuracy %</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n"/>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
+      <c r="E16" s="13" t="n"/>
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="G16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="I16" s="17" t="inlineStr">
+      <c r="I16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="J16" s="16" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="K16" s="17" t="inlineStr">
+      <c r="K16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="L16" s="16" t="inlineStr">
-        <is>
-          <t>9/10</t>
-        </is>
-      </c>
-      <c r="M16" s="18" t="inlineStr">
-        <is>
-          <t>90.0%</t>
-        </is>
-      </c>
-      <c r="N16" s="16" t="inlineStr">
+      <c r="L16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="O16" s="17" t="inlineStr">
+      <c r="M16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="P16" s="16" t="inlineStr">
+      <c r="N16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="Q16" s="17" t="inlineStr">
+      <c r="O16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="R16" s="16" t="inlineStr">
+      <c r="P16" s="14" t="inlineStr">
         <is>
           <t>10/10</t>
         </is>
       </c>
-      <c r="S16" s="17" t="inlineStr">
+      <c r="Q16" s="15" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="R16" s="14" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="S16" s="15" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>All Correct</t>
         </is>
       </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>9 / 10  (90.0%)</t>
+      <c r="F17" s="17" t="inlineStr">
+        <is>
+          <t>10 / 10  (100.0%)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>Legend:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  </t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="20" t="inlineStr">
         <is>
           <t>Correct prediction</t>
         </is>
       </c>
-      <c r="C20" s="24" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  </t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="20" t="inlineStr">
         <is>
           <t>Wrong prediction</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">  </t>
         </is>
       </c>
-      <c r="F20" s="23" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>Ground truth value</t>
         </is>
       </c>
-      <c r="G20" s="26" t="inlineStr">
+      <c r="G20" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  </t>
         </is>
       </c>
-      <c r="H20" s="23" t="inlineStr">
+      <c r="H20" s="20" t="inlineStr">
         <is>
           <t>All vitals correct</t>
         </is>
       </c>
-      <c r="I20" s="27" t="inlineStr">
+      <c r="I20" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  </t>
         </is>
       </c>
-      <c r="J20" s="23" t="inlineStr">
+      <c r="J20" s="20" t="inlineStr">
         <is>
           <t>Some vitals wrong</t>
         </is>

</xml_diff>